<commit_message>
feat: adding june data and try some splits
</commit_message>
<xml_diff>
--- a/data/bps_2022_2026.xlsx
+++ b/data/bps_2022_2026.xlsx
@@ -654,8 +654,11 @@
       <c r="H8" t="str">
         <v>137830116.83</v>
       </c>
+      <c r="I8" t="str">
+        <v>188842935.12</v>
+      </c>
       <c r="P8" t="str">
-        <v>724412064.33</v>
+        <v>913254999.46</v>
       </c>
     </row>
     <row r="9">
@@ -822,7 +825,7 @@
         <v>71675388.41</v>
       </c>
       <c r="L12" t="str">
-        <v>72943350.17</v>
+        <v>72943350.16</v>
       </c>
       <c r="M12" t="str">
         <v>98284124.04</v>
@@ -856,8 +859,11 @@
       <c r="H13" t="str">
         <v>89961375.48</v>
       </c>
+      <c r="I13" t="str">
+        <v>93897013.51</v>
+      </c>
       <c r="P13" t="str">
-        <v>408403900.53</v>
+        <v>502300914.04</v>
       </c>
     </row>
     <row r="14">
@@ -1058,8 +1064,11 @@
       <c r="H18" t="str">
         <v>245806272.04</v>
       </c>
+      <c r="I18" t="str">
+        <v>235935967.33</v>
+      </c>
       <c r="P18" t="str">
-        <v>1616955469.51</v>
+        <v>1852891436.83</v>
       </c>
     </row>
     <row r="19">
@@ -1260,8 +1269,11 @@
       <c r="H23" t="str">
         <v>144225788.31</v>
       </c>
+      <c r="I23" t="str">
+        <v>172267358.31</v>
+      </c>
       <c r="P23" t="str">
-        <v>883155082.05</v>
+        <v>1055422440.36</v>
       </c>
     </row>
     <row r="24">
@@ -1462,8 +1474,11 @@
       <c r="H28" t="str">
         <v>199862641.57</v>
       </c>
+      <c r="I28" t="str">
+        <v>165683227.43</v>
+      </c>
       <c r="P28" t="str">
-        <v>983852463.41</v>
+        <v>1149535690.85</v>
       </c>
     </row>
     <row r="29">
@@ -1486,7 +1501,7 @@
         <v>5234175433.30</v>
       </c>
       <c r="I29" t="str">
-        <v>4101537721.63</v>
+        <v>4958164223.32</v>
       </c>
       <c r="J29" t="str">
         <v>4222970193.02</v>
@@ -1507,7 +1522,7 @@
         <v>4947743817.75</v>
       </c>
       <c r="P29" t="str">
-        <v>56592573255.76</v>
+        <v>57449199757.46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>